<commit_message>
Fill in shadow prices for binding constraints (carrot and mesclun bed caps)
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h0015\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h0015\Heekum-Kim\capabilities\marginal-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B2E4590-EE2C-4433-ABCA-11F91CF8B1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790C0574-3A2B-471B-946F-6026D49F1131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -67,6 +67,7 @@
     <definedName name="solver_drv" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">Inputs!$B$6:$B$8</definedName>
@@ -82,12 +83,15 @@
     <definedName name="solver_msl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_num" localSheetId="2" hidden="1">6</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Inputs!$B$31</definedName>
     <definedName name="solver_opt" localSheetId="2" hidden="1">Optimization!$B$31</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Results!$G$8</definedName>
     <definedName name="solver_pre" localSheetId="2" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
@@ -113,10 +117,13 @@
     <definedName name="solver_tol" localSheetId="2" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="TEMP_HRS_EACH">Inputs!$B$30</definedName>
     <definedName name="TEMP_MAX">Inputs!$B$29</definedName>
     <definedName name="TEMP_MAX_SHADOW">Results!$B$22</definedName>
@@ -877,15 +884,15 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1301,7 +1308,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>13</v>
@@ -3666,37 +3673,37 @@
         <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="J25" s="13" t="str">
+      <c r="J25" s="13">
         <f>IF(21&lt;=CAR_MAXBED,21,"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="14" t="str">
+        <v>21</v>
+      </c>
+      <c r="K25" s="14">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="L25" s="15" t="str">
+        <v>1058.1365663175229</v>
+      </c>
+      <c r="L25" s="15">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="M25" s="16" t="str">
+        <v>30870.426498568107</v>
+      </c>
+      <c r="M25" s="16">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="N25" s="15" t="str">
+        <v>9240</v>
+      </c>
+      <c r="N25" s="15">
         <f t="shared" si="9"/>
-        <v/>
-      </c>
-      <c r="O25" s="16" t="str">
+        <v>40110.426498568107</v>
+      </c>
+      <c r="O25" s="16">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="P25" s="15" t="str">
+        <v>43974</v>
+      </c>
+      <c r="P25" s="15">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="Q25" s="15" t="str">
+        <v>3863.5735014318925</v>
+      </c>
+      <c r="Q25" s="15">
         <f t="shared" si="19"/>
-        <v/>
+        <v>1741.5052455431578</v>
       </c>
       <c r="R25" s="13">
         <f>IF(21&lt;=MES_MAXBED,21,"")</f>
@@ -5179,11 +5186,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="41.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
@@ -5200,7 +5207,9 @@
       <c r="A18" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B18" s="23"/>
+      <c r="B18" s="23">
+        <v>0</v>
+      </c>
       <c r="C18" s="18" t="s">
         <v>148</v>
       </c>
@@ -5209,7 +5218,9 @@
       <c r="A19" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B19" s="23"/>
+      <c r="B19" s="23">
+        <v>352.5</v>
+      </c>
       <c r="C19" s="18" t="s">
         <v>150</v>
       </c>
@@ -5218,7 +5229,9 @@
       <c r="A20" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="23"/>
+      <c r="B20" s="23">
+        <v>246.48</v>
+      </c>
       <c r="C20" s="18" t="s">
         <v>152</v>
       </c>
@@ -5227,7 +5240,9 @@
       <c r="A21" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="23">
+        <v>0</v>
+      </c>
       <c r="C21" s="18" t="s">
         <v>154</v>
       </c>
@@ -5236,7 +5251,9 @@
       <c r="A22" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B22" s="23"/>
+      <c r="B22" s="23">
+        <v>0</v>
+      </c>
       <c r="C22" s="18" t="s">
         <v>156</v>
       </c>
@@ -5284,7 +5301,7 @@
       <c r="D4" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E4" s="27"/>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
@@ -5424,7 +5441,7 @@
       <c r="A17" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="B17" s="30" t="s">
+      <c r="B17" s="28" t="s">
         <v>180</v>
       </c>
       <c r="C17" s="6">
@@ -5438,7 +5455,7 @@
       <c r="A18" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="27" t="s">
         <v>191</v>
       </c>
       <c r="C18" s="6">
@@ -5449,12 +5466,12 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="21" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">

</xml_diff>

<commit_message>
Add Figures sheet to model.xlsx with MC vs price series for figures 1 and 2
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h0015\Heekum-Kim\capabilities\marginal-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790C0574-3A2B-471B-946F-6026D49F1131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C84F43E-9708-4A7F-9358-E8F3476352AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Cost &amp; Marginal Cost" sheetId="2" r:id="rId2"/>
     <sheet name="Optimization" sheetId="3" r:id="rId3"/>
     <sheet name="Results" sheetId="4" r:id="rId4"/>
-    <sheet name="Checks" sheetId="5" r:id="rId5"/>
+    <sheet name="Figures" sheetId="6" r:id="rId5"/>
+    <sheet name="Checks" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="CAR_BEDS">Optimization!$B$7</definedName>
@@ -165,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="197">
   <si>
     <t>Inputs — the named contract</t>
   </si>
@@ -741,20 +742,36 @@
   </si>
   <si>
     <t>'10/20/30</t>
+  </si>
+  <si>
+    <t>Beds</t>
+  </si>
+  <si>
+    <t>Tomato MC</t>
+  </si>
+  <si>
+    <t>Tomato price</t>
+  </si>
+  <si>
+    <t>Carrot MC</t>
+  </si>
+  <si>
+    <t>Carrot price</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="\$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0000"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -811,6 +828,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -850,10 +874,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -887,14 +912,16 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -976,6 +1003,2745 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Tomato marginal cost vs price</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Figures!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tomato MC</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Figures!$A$2:$A$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Figures!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>4317.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5795.6250000000036</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6703.125</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7660.859375</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4906.2750000000051</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5585.7089062500017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6360.7668437500033</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7243.7792796875074</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8248.586534375012</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9390.7174472031256</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10687.588677253138</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12158.726978841107</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13826.017053974152</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15713.977874345364</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17850.070688251115</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20265.042286194512</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>22993.307496844121</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>26073.375326761772</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>29548.323647694342</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5DA3-434F-9DCD-B6C07349197E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Figures!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tomato price</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Figures!$A$2:$A$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Figures!$C$2:$C$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5DA3-434F-9DCD-B6C07349197E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1810372751"/>
+        <c:axId val="1506675311"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1810372751"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Beds</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> planted</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1506675311"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1506675311"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Dollars</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> per bed</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1810372751"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Carrot marginal cost vs</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> price</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Figures!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Carrot MC</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Figures!$D$2:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Figures!$E$2:$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1507.7083333333333</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1561.0937499999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1616.481119791667</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1673.9371744791652</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1733.530731201171</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1795.332755025227</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1859.4164233334868</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1925.8571920852646</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1994.7328640100477</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2066.1236587860258</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2140.1122852607878</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2216.7840157725441</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2296.2267626316061</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2378.5311568237667</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2463.7906289988823</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2552.1014928097429</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1670.9013431626554</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1589.1387909931072</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1638.1753169880685</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1688.9454575384007</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E91F-44F4-8D48-54C35125A68C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Figures!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Carrot price</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Figures!$D$2:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Figures!$F$2:$F$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2094</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E91F-44F4-8D48-54C35125A68C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1012906048"/>
+        <c:axId val="920895312"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1012906048"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Beds</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Planted</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="920895312"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="920895312"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>dollars per bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1012906048"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>41775</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>117222</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>379161</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>142039</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC93E75D-E9EF-F7BD-1230-23D1309D77B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>509671</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>70017</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>620713</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>108618</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDBD08A7-B636-A179-2AED-07CE8257A587}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5268,6 +8034,521 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DEEBEE8-C51F-4F11-AF1F-DD0E88D764A6}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="3" width="13.796875" customWidth="1"/>
+    <col min="5" max="5" width="13.9296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="29">
+        <f>'Cost &amp; Marginal Cost'!I5</f>
+        <v>4317.5</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C21" si="0">TOM_PRICE</f>
+        <v>8800</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q5</f>
+        <v>1507.7083333333333</v>
+      </c>
+      <c r="F2">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="29">
+        <f>'Cost &amp; Marginal Cost'!I6</f>
+        <v>5005</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q6</f>
+        <v>1561.0937499999998</v>
+      </c>
+      <c r="F3">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="29">
+        <f>'Cost &amp; Marginal Cost'!I7</f>
+        <v>5795.6250000000036</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q7</f>
+        <v>1616.481119791667</v>
+      </c>
+      <c r="F4">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="29">
+        <f>'Cost &amp; Marginal Cost'!I8</f>
+        <v>6703.125</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q8</f>
+        <v>1673.9371744791652</v>
+      </c>
+      <c r="F5">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="29">
+        <f>'Cost &amp; Marginal Cost'!I9</f>
+        <v>7660.859375</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q9</f>
+        <v>1733.530731201171</v>
+      </c>
+      <c r="F6">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="29">
+        <f>'Cost &amp; Marginal Cost'!I10</f>
+        <v>4906.2750000000051</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q10</f>
+        <v>1795.332755025227</v>
+      </c>
+      <c r="F7">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="29">
+        <f>'Cost &amp; Marginal Cost'!I11</f>
+        <v>5585.7089062500017</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q11</f>
+        <v>1859.4164233334868</v>
+      </c>
+      <c r="F8">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="29">
+        <f>'Cost &amp; Marginal Cost'!I12</f>
+        <v>6360.7668437500033</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q12</f>
+        <v>1925.8571920852646</v>
+      </c>
+      <c r="F9">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="29">
+        <f>'Cost &amp; Marginal Cost'!I13</f>
+        <v>7243.7792796875074</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q13</f>
+        <v>1994.7328640100477</v>
+      </c>
+      <c r="F10">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="29">
+        <f>'Cost &amp; Marginal Cost'!I14</f>
+        <v>8248.586534375012</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
+      </c>
+      <c r="E11" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q14</f>
+        <v>2066.1236587860258</v>
+      </c>
+      <c r="F11">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="29">
+        <f>'Cost &amp; Marginal Cost'!I15</f>
+        <v>9390.7174472031256</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q15</f>
+        <v>2140.1122852607878</v>
+      </c>
+      <c r="F12">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="29">
+        <f>'Cost &amp; Marginal Cost'!I16</f>
+        <v>10687.588677253138</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
+      <c r="E13" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q16</f>
+        <v>2216.7840157725441</v>
+      </c>
+      <c r="F13">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="29">
+        <f>'Cost &amp; Marginal Cost'!I17</f>
+        <v>12158.726978841107</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q17</f>
+        <v>2296.2267626316061</v>
+      </c>
+      <c r="F14">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="29">
+        <f>'Cost &amp; Marginal Cost'!I18</f>
+        <v>13826.017053974152</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q18</f>
+        <v>2378.5311568237667</v>
+      </c>
+      <c r="F15">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="29">
+        <f>'Cost &amp; Marginal Cost'!I19</f>
+        <v>15713.977874345364</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q19</f>
+        <v>2463.7906289988823</v>
+      </c>
+      <c r="F16">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="29">
+        <f>'Cost &amp; Marginal Cost'!I20</f>
+        <v>17850.070688251115</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="E17" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q20</f>
+        <v>2552.1014928097429</v>
+      </c>
+      <c r="F17">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="29">
+        <f>'Cost &amp; Marginal Cost'!I21</f>
+        <v>20265.042286194512</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q21</f>
+        <v>1670.9013431626554</v>
+      </c>
+      <c r="F18">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="29">
+        <f>'Cost &amp; Marginal Cost'!I22</f>
+        <v>22993.307496844121</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D19">
+        <v>18</v>
+      </c>
+      <c r="E19" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q22</f>
+        <v>1589.1387909931072</v>
+      </c>
+      <c r="F19">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="29">
+        <f>'Cost &amp; Marginal Cost'!I23</f>
+        <v>26073.375326761772</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q23</f>
+        <v>1638.1753169880685</v>
+      </c>
+      <c r="F20">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="29">
+        <f>'Cost &amp; Marginal Cost'!I24</f>
+        <v>29548.323647694342</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21" s="29">
+        <f>'Cost &amp; Marginal Cost'!Q24</f>
+        <v>1688.9454575384007</v>
+      </c>
+      <c r="F21">
+        <f>CAR_PRICE</f>
+        <v>2094</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -5466,12 +8747,12 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
     </row>
     <row r="21" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">

</xml_diff>